<commit_message>
Local smoke test  identified bugfixes
</commit_message>
<xml_diff>
--- a/docs/admin-frontend-qa-checklist-local-env.xlsx
+++ b/docs/admin-frontend-qa-checklist-local-env.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayanc\OneDrive\Desktop\cabbo-frontends\cabbo-admin-frontend\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd80ce77b79934dc/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6982CC3B-DFAC-4EDA-9416-6BCCC8259F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{A72889CB-7753-4260-9A19-C81F8BF0DA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17549F2E-096A-4B8C-96CB-77EC66C9DCB6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="441">
   <si>
     <t>Admin Frontend QA Checklist - Local Environment</t>
   </si>
@@ -537,21 +537,6 @@
     <t>Only matching statuses appear and empty states behave correctly.</t>
   </si>
   <si>
-    <t>LOC-029</t>
-  </si>
-  <si>
-    <t>Search/debounce</t>
-  </si>
-  <si>
-    <t>Type search text quickly and clear it.</t>
-  </si>
-  <si>
-    <t>Debounced query behaves predictably; clear returns default results.</t>
-  </si>
-  <si>
-    <t>Searchable bookings</t>
-  </si>
-  <si>
     <t>LOC-030</t>
   </si>
   <si>
@@ -588,9 +573,6 @@
     <t>Open detail from card</t>
   </si>
   <si>
-    <t>Click a trip card/detail link.</t>
-  </si>
-  <si>
     <t>Booking detail route opens with the selected booking data.</t>
   </si>
   <si>
@@ -1360,6 +1342,9 @@
   </si>
   <si>
     <t>Swaroop C</t>
+  </si>
+  <si>
+    <t>Click a trip card/open button link.</t>
   </si>
 </sst>
 </file>
@@ -1392,7 +1377,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1408,6 +1393,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEFF6FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1439,7 +1430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1450,6 +1441,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1833,8 +1827,8 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <f>COUNTA(Checklist!A2:A81)</f>
-        <v>80</v>
+        <f>COUNTA(Checklist!A2:A80)</f>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -1842,8 +1836,8 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <f>COUNTIF(Checklist!H2:H81,"Pass")</f>
-        <v>0</v>
+        <f>COUNTIF(Checklist!H2:H80,"Pass")</f>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -1851,7 +1845,7 @@
         <v>11</v>
       </c>
       <c r="B8">
-        <f>COUNTIF(Checklist!H2:H81,"Fail")</f>
+        <f>COUNTIF(Checklist!H2:H80,"Fail")</f>
         <v>0</v>
       </c>
     </row>
@@ -1860,7 +1854,7 @@
         <v>12</v>
       </c>
       <c r="B9">
-        <f>COUNTIF(Checklist!H2:H81,"Blocked")</f>
+        <f>COUNTIF(Checklist!H2:H80,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -1869,7 +1863,7 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <f>COUNTIF(Checklist!H2:H81,"N/A")</f>
+        <f>COUNTIF(Checklist!H2:H80,"N/A")</f>
         <v>0</v>
       </c>
     </row>
@@ -1878,8 +1872,8 @@
         <v>14</v>
       </c>
       <c r="B11">
-        <f>COUNTIF(Checklist!H2:H81,"Not Started")</f>
-        <v>80</v>
+        <f>COUNTIF(Checklist!H2:H80,"Not Started")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -1888,7 +1882,7 @@
       </c>
       <c r="B12">
         <f>IF(B6=0,0,(B7+B10)/B6)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1899,7 +1893,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:K80"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1972,11 +1966,11 @@
       <c r="G2" t="s">
         <v>33</v>
       </c>
-      <c r="H2" t="s">
-        <v>14</v>
+      <c r="H2" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2001,11 +1995,11 @@
       <c r="G3" t="s">
         <v>38</v>
       </c>
-      <c r="H3" t="s">
-        <v>14</v>
+      <c r="H3" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2030,11 +2024,11 @@
       <c r="G4" t="s">
         <v>43</v>
       </c>
-      <c r="H4" t="s">
-        <v>14</v>
+      <c r="H4" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2059,11 +2053,11 @@
       <c r="G5" t="s">
         <v>48</v>
       </c>
-      <c r="H5" t="s">
-        <v>14</v>
+      <c r="H5" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2088,11 +2082,11 @@
       <c r="G6" t="s">
         <v>48</v>
       </c>
-      <c r="H6" t="s">
-        <v>14</v>
+      <c r="H6" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2117,11 +2111,11 @@
       <c r="G7" t="s">
         <v>59</v>
       </c>
-      <c r="H7" t="s">
-        <v>14</v>
+      <c r="H7" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2146,11 +2140,11 @@
       <c r="G8" t="s">
         <v>64</v>
       </c>
-      <c r="H8" t="s">
-        <v>14</v>
+      <c r="H8" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2175,11 +2169,11 @@
       <c r="G9" t="s">
         <v>69</v>
       </c>
-      <c r="H9" t="s">
-        <v>14</v>
+      <c r="H9" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2204,11 +2198,11 @@
       <c r="G10" t="s">
         <v>59</v>
       </c>
-      <c r="H10" t="s">
-        <v>14</v>
+      <c r="H10" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2233,11 +2227,11 @@
       <c r="G11" t="s">
         <v>78</v>
       </c>
-      <c r="H11" t="s">
-        <v>14</v>
+      <c r="H11" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2262,11 +2256,11 @@
       <c r="G12" t="s">
         <v>78</v>
       </c>
-      <c r="H12" t="s">
-        <v>14</v>
+      <c r="H12" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2291,11 +2285,11 @@
       <c r="G13" t="s">
         <v>87</v>
       </c>
-      <c r="H13" t="s">
-        <v>14</v>
+      <c r="H13" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2320,11 +2314,11 @@
       <c r="G14" t="s">
         <v>93</v>
       </c>
-      <c r="H14" t="s">
-        <v>14</v>
+      <c r="H14" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2349,11 +2343,11 @@
       <c r="G15" t="s">
         <v>98</v>
       </c>
-      <c r="H15" t="s">
-        <v>14</v>
+      <c r="H15" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2378,11 +2372,11 @@
       <c r="G16" t="s">
         <v>104</v>
       </c>
-      <c r="H16" t="s">
-        <v>14</v>
+      <c r="H16" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2407,11 +2401,11 @@
       <c r="G17" t="s">
         <v>110</v>
       </c>
-      <c r="H17" t="s">
-        <v>14</v>
+      <c r="H17" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2436,11 +2430,11 @@
       <c r="G18" t="s">
         <v>115</v>
       </c>
-      <c r="H18" t="s">
-        <v>14</v>
+      <c r="H18" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2465,11 +2459,11 @@
       <c r="G19" t="s">
         <v>120</v>
       </c>
-      <c r="H19" t="s">
-        <v>14</v>
+      <c r="H19" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2494,11 +2488,11 @@
       <c r="G20" t="s">
         <v>125</v>
       </c>
-      <c r="H20" t="s">
-        <v>14</v>
+      <c r="H20" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2523,11 +2517,11 @@
       <c r="G21" t="s">
         <v>130</v>
       </c>
-      <c r="H21" t="s">
-        <v>14</v>
+      <c r="H21" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2552,11 +2546,11 @@
       <c r="G22" t="s">
         <v>130</v>
       </c>
-      <c r="H22" t="s">
-        <v>14</v>
+      <c r="H22" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2581,11 +2575,11 @@
       <c r="G23" t="s">
         <v>140</v>
       </c>
-      <c r="H23" t="s">
-        <v>14</v>
+      <c r="H23" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2610,11 +2604,11 @@
       <c r="G24" t="s">
         <v>145</v>
       </c>
-      <c r="H24" t="s">
-        <v>14</v>
+      <c r="H24" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2639,11 +2633,11 @@
       <c r="G25" t="s">
         <v>150</v>
       </c>
-      <c r="H25" t="s">
-        <v>14</v>
+      <c r="H25" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2668,11 +2662,11 @@
       <c r="G26" t="s">
         <v>155</v>
       </c>
-      <c r="H26" t="s">
-        <v>14</v>
+      <c r="H26" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2697,11 +2691,11 @@
       <c r="G27" t="s">
         <v>161</v>
       </c>
-      <c r="H27" t="s">
-        <v>14</v>
+      <c r="H27" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2726,11 +2720,11 @@
       <c r="G28" t="s">
         <v>166</v>
       </c>
-      <c r="H28" t="s">
-        <v>14</v>
+      <c r="H28" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2755,11 +2749,11 @@
       <c r="G29" t="s">
         <v>140</v>
       </c>
-      <c r="H29" t="s">
-        <v>14</v>
+      <c r="H29" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2784,11 +2778,11 @@
       <c r="G30" t="s">
         <v>175</v>
       </c>
-      <c r="H30" t="s">
-        <v>14</v>
+      <c r="H30" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2811,42 +2805,42 @@
         <v>53</v>
       </c>
       <c r="G31" t="s">
-        <v>180</v>
-      </c>
-      <c r="H31" t="s">
-        <v>14</v>
+        <v>175</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
+        <v>180</v>
+      </c>
+      <c r="B32" t="s">
         <v>181</v>
-      </c>
-      <c r="B32" t="s">
-        <v>157</v>
       </c>
       <c r="C32" t="s">
         <v>182</v>
       </c>
       <c r="D32" t="s">
+        <v>440</v>
+      </c>
+      <c r="E32" t="s">
         <v>183</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
+        <v>32</v>
+      </c>
+      <c r="G32" t="s">
         <v>184</v>
       </c>
-      <c r="F32" t="s">
-        <v>53</v>
-      </c>
-      <c r="G32" t="s">
-        <v>180</v>
-      </c>
-      <c r="H32" t="s">
-        <v>14</v>
+      <c r="H32" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -2854,181 +2848,181 @@
         <v>185</v>
       </c>
       <c r="B33" t="s">
+        <v>181</v>
+      </c>
+      <c r="C33" t="s">
         <v>186</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>187</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>188</v>
-      </c>
-      <c r="E33" t="s">
-        <v>189</v>
       </c>
       <c r="F33" t="s">
         <v>32</v>
       </c>
       <c r="G33" t="s">
-        <v>190</v>
-      </c>
-      <c r="H33" t="s">
-        <v>14</v>
+        <v>189</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
+        <v>190</v>
+      </c>
+      <c r="B34" t="s">
+        <v>181</v>
+      </c>
+      <c r="C34" t="s">
         <v>191</v>
       </c>
-      <c r="B34" t="s">
-        <v>186</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>192</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>193</v>
-      </c>
-      <c r="E34" t="s">
-        <v>194</v>
       </c>
       <c r="F34" t="s">
         <v>32</v>
       </c>
       <c r="G34" t="s">
-        <v>195</v>
-      </c>
-      <c r="H34" t="s">
-        <v>14</v>
+        <v>194</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
+        <v>195</v>
+      </c>
+      <c r="B35" t="s">
+        <v>181</v>
+      </c>
+      <c r="C35" t="s">
         <v>196</v>
       </c>
-      <c r="B35" t="s">
-        <v>186</v>
-      </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>197</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>198</v>
-      </c>
-      <c r="E35" t="s">
-        <v>199</v>
       </c>
       <c r="F35" t="s">
         <v>32</v>
       </c>
       <c r="G35" t="s">
-        <v>200</v>
-      </c>
-      <c r="H35" t="s">
-        <v>14</v>
+        <v>199</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
+        <v>200</v>
+      </c>
+      <c r="B36" t="s">
+        <v>181</v>
+      </c>
+      <c r="C36" t="s">
         <v>201</v>
       </c>
-      <c r="B36" t="s">
-        <v>186</v>
-      </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>202</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>203</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
+        <v>53</v>
+      </c>
+      <c r="G36" t="s">
         <v>204</v>
       </c>
-      <c r="F36" t="s">
-        <v>32</v>
-      </c>
-      <c r="G36" t="s">
-        <v>205</v>
-      </c>
-      <c r="H36" t="s">
-        <v>14</v>
+      <c r="H36" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
+        <v>205</v>
+      </c>
+      <c r="B37" t="s">
+        <v>181</v>
+      </c>
+      <c r="C37" t="s">
         <v>206</v>
       </c>
-      <c r="B37" t="s">
-        <v>186</v>
-      </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>207</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>208</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
+        <v>32</v>
+      </c>
+      <c r="G37" t="s">
         <v>209</v>
       </c>
-      <c r="F37" t="s">
-        <v>53</v>
-      </c>
-      <c r="G37" t="s">
-        <v>210</v>
-      </c>
-      <c r="H37" t="s">
-        <v>14</v>
+      <c r="H37" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
+        <v>210</v>
+      </c>
+      <c r="B38" t="s">
+        <v>181</v>
+      </c>
+      <c r="C38" t="s">
         <v>211</v>
       </c>
-      <c r="B38" t="s">
-        <v>186</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>212</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>213</v>
-      </c>
-      <c r="E38" t="s">
-        <v>214</v>
       </c>
       <c r="F38" t="s">
         <v>32</v>
       </c>
       <c r="G38" t="s">
-        <v>215</v>
-      </c>
-      <c r="H38" t="s">
-        <v>14</v>
+        <v>214</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
+        <v>215</v>
+      </c>
+      <c r="B39" t="s">
         <v>216</v>
-      </c>
-      <c r="B39" t="s">
-        <v>186</v>
       </c>
       <c r="C39" t="s">
         <v>217</v>
@@ -3045,11 +3039,11 @@
       <c r="G39" t="s">
         <v>220</v>
       </c>
-      <c r="H39" t="s">
-        <v>14</v>
+      <c r="H39" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3057,123 +3051,123 @@
         <v>221</v>
       </c>
       <c r="B40" t="s">
+        <v>216</v>
+      </c>
+      <c r="C40" t="s">
         <v>222</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>223</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>224</v>
-      </c>
-      <c r="E40" t="s">
-        <v>225</v>
       </c>
       <c r="F40" t="s">
         <v>32</v>
       </c>
       <c r="G40" t="s">
-        <v>226</v>
-      </c>
-      <c r="H40" t="s">
-        <v>14</v>
+        <v>225</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
+        <v>226</v>
+      </c>
+      <c r="B41" t="s">
+        <v>216</v>
+      </c>
+      <c r="C41" t="s">
         <v>227</v>
       </c>
-      <c r="B41" t="s">
-        <v>222</v>
-      </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>228</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>229</v>
-      </c>
-      <c r="E41" t="s">
-        <v>230</v>
       </c>
       <c r="F41" t="s">
         <v>32</v>
       </c>
       <c r="G41" t="s">
-        <v>231</v>
-      </c>
-      <c r="H41" t="s">
-        <v>14</v>
+        <v>230</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
+        <v>231</v>
+      </c>
+      <c r="B42" t="s">
+        <v>216</v>
+      </c>
+      <c r="C42" t="s">
         <v>232</v>
       </c>
-      <c r="B42" t="s">
-        <v>222</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>233</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>234</v>
-      </c>
-      <c r="E42" t="s">
-        <v>235</v>
       </c>
       <c r="F42" t="s">
         <v>32</v>
       </c>
       <c r="G42" t="s">
-        <v>236</v>
-      </c>
-      <c r="H42" t="s">
-        <v>14</v>
+        <v>235</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
+        <v>236</v>
+      </c>
+      <c r="B43" t="s">
+        <v>216</v>
+      </c>
+      <c r="C43" t="s">
         <v>237</v>
       </c>
-      <c r="B43" t="s">
-        <v>222</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>238</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>239</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
+        <v>53</v>
+      </c>
+      <c r="G43" t="s">
         <v>240</v>
       </c>
-      <c r="F43" t="s">
-        <v>32</v>
-      </c>
-      <c r="G43" t="s">
-        <v>241</v>
-      </c>
-      <c r="H43" t="s">
-        <v>14</v>
+      <c r="H43" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
+        <v>241</v>
+      </c>
+      <c r="B44" t="s">
         <v>242</v>
-      </c>
-      <c r="B44" t="s">
-        <v>222</v>
       </c>
       <c r="C44" t="s">
         <v>243</v>
@@ -3185,16 +3179,16 @@
         <v>245</v>
       </c>
       <c r="F44" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="G44" t="s">
         <v>246</v>
       </c>
-      <c r="H44" t="s">
-        <v>14</v>
+      <c r="H44" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3202,144 +3196,144 @@
         <v>247</v>
       </c>
       <c r="B45" t="s">
+        <v>242</v>
+      </c>
+      <c r="C45" t="s">
         <v>248</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>249</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>250</v>
-      </c>
-      <c r="E45" t="s">
-        <v>251</v>
       </c>
       <c r="F45" t="s">
         <v>32</v>
       </c>
       <c r="G45" t="s">
-        <v>252</v>
-      </c>
-      <c r="H45" t="s">
-        <v>14</v>
+        <v>251</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
+        <v>252</v>
+      </c>
+      <c r="B46" t="s">
+        <v>242</v>
+      </c>
+      <c r="C46" t="s">
         <v>253</v>
       </c>
-      <c r="B46" t="s">
-        <v>248</v>
-      </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>254</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>255</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
+        <v>53</v>
+      </c>
+      <c r="G46" t="s">
         <v>256</v>
       </c>
-      <c r="F46" t="s">
-        <v>32</v>
-      </c>
-      <c r="G46" t="s">
-        <v>257</v>
-      </c>
-      <c r="H46" t="s">
-        <v>14</v>
+      <c r="H46" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
+        <v>257</v>
+      </c>
+      <c r="B47" t="s">
+        <v>242</v>
+      </c>
+      <c r="C47" t="s">
         <v>258</v>
       </c>
-      <c r="B47" t="s">
-        <v>248</v>
-      </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>259</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>260</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
+        <v>32</v>
+      </c>
+      <c r="G47" t="s">
         <v>261</v>
       </c>
-      <c r="F47" t="s">
-        <v>53</v>
-      </c>
-      <c r="G47" t="s">
-        <v>262</v>
-      </c>
-      <c r="H47" t="s">
-        <v>14</v>
+      <c r="H47" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
+        <v>262</v>
+      </c>
+      <c r="B48" t="s">
+        <v>242</v>
+      </c>
+      <c r="C48" t="s">
         <v>263</v>
       </c>
-      <c r="B48" t="s">
-        <v>248</v>
-      </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>264</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>265</v>
       </c>
-      <c r="E48" t="s">
-        <v>266</v>
-      </c>
       <c r="F48" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="G48" t="s">
-        <v>267</v>
-      </c>
-      <c r="H48" t="s">
-        <v>14</v>
+        <v>256</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
+        <v>266</v>
+      </c>
+      <c r="B49" t="s">
+        <v>267</v>
+      </c>
+      <c r="C49" t="s">
         <v>268</v>
       </c>
-      <c r="B49" t="s">
-        <v>248</v>
-      </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>269</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>270</v>
       </c>
-      <c r="E49" t="s">
+      <c r="F49" t="s">
+        <v>32</v>
+      </c>
+      <c r="G49" t="s">
         <v>271</v>
       </c>
-      <c r="F49" t="s">
-        <v>53</v>
-      </c>
-      <c r="G49" t="s">
-        <v>262</v>
-      </c>
-      <c r="H49" t="s">
-        <v>14</v>
+      <c r="H49" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3347,123 +3341,123 @@
         <v>272</v>
       </c>
       <c r="B50" t="s">
+        <v>267</v>
+      </c>
+      <c r="C50" t="s">
         <v>273</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>274</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>275</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
+        <v>53</v>
+      </c>
+      <c r="G50" t="s">
         <v>276</v>
       </c>
-      <c r="F50" t="s">
-        <v>32</v>
-      </c>
-      <c r="G50" t="s">
-        <v>277</v>
-      </c>
-      <c r="H50" t="s">
-        <v>14</v>
+      <c r="H50" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
+        <v>277</v>
+      </c>
+      <c r="B51" t="s">
+        <v>267</v>
+      </c>
+      <c r="C51" t="s">
         <v>278</v>
       </c>
-      <c r="B51" t="s">
-        <v>273</v>
-      </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>279</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>280</v>
       </c>
-      <c r="E51" t="s">
-        <v>281</v>
-      </c>
       <c r="F51" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="G51" t="s">
-        <v>282</v>
-      </c>
-      <c r="H51" t="s">
-        <v>14</v>
+        <v>251</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
+        <v>281</v>
+      </c>
+      <c r="B52" t="s">
+        <v>267</v>
+      </c>
+      <c r="C52" t="s">
+        <v>282</v>
+      </c>
+      <c r="D52" t="s">
         <v>283</v>
       </c>
-      <c r="B52" t="s">
-        <v>273</v>
-      </c>
-      <c r="C52" t="s">
+      <c r="E52" t="s">
         <v>284</v>
-      </c>
-      <c r="D52" t="s">
-        <v>285</v>
-      </c>
-      <c r="E52" t="s">
-        <v>286</v>
       </c>
       <c r="F52" t="s">
         <v>32</v>
       </c>
       <c r="G52" t="s">
-        <v>257</v>
-      </c>
-      <c r="H52" t="s">
-        <v>14</v>
+        <v>261</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
+        <v>285</v>
+      </c>
+      <c r="B53" t="s">
+        <v>267</v>
+      </c>
+      <c r="C53" t="s">
+        <v>286</v>
+      </c>
+      <c r="D53" t="s">
         <v>287</v>
       </c>
-      <c r="B53" t="s">
-        <v>273</v>
-      </c>
-      <c r="C53" t="s">
+      <c r="E53" t="s">
         <v>288</v>
       </c>
-      <c r="D53" t="s">
+      <c r="F53" t="s">
+        <v>53</v>
+      </c>
+      <c r="G53" t="s">
         <v>289</v>
       </c>
-      <c r="E53" t="s">
-        <v>290</v>
-      </c>
-      <c r="F53" t="s">
-        <v>32</v>
-      </c>
-      <c r="G53" t="s">
-        <v>267</v>
-      </c>
-      <c r="H53" t="s">
-        <v>14</v>
+      <c r="H53" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
+        <v>290</v>
+      </c>
+      <c r="B54" t="s">
         <v>291</v>
-      </c>
-      <c r="B54" t="s">
-        <v>273</v>
       </c>
       <c r="C54" t="s">
         <v>292</v>
@@ -3475,16 +3469,16 @@
         <v>294</v>
       </c>
       <c r="F54" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="G54" t="s">
         <v>295</v>
       </c>
-      <c r="H54" t="s">
-        <v>14</v>
+      <c r="H54" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3492,115 +3486,115 @@
         <v>296</v>
       </c>
       <c r="B55" t="s">
+        <v>291</v>
+      </c>
+      <c r="C55" t="s">
         <v>297</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
         <v>298</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>299</v>
-      </c>
-      <c r="E55" t="s">
-        <v>300</v>
       </c>
       <c r="F55" t="s">
         <v>32</v>
       </c>
       <c r="G55" t="s">
-        <v>301</v>
-      </c>
-      <c r="H55" t="s">
-        <v>14</v>
+        <v>300</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
+        <v>301</v>
+      </c>
+      <c r="B56" t="s">
+        <v>291</v>
+      </c>
+      <c r="C56" t="s">
         <v>302</v>
       </c>
-      <c r="B56" t="s">
-        <v>297</v>
-      </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
         <v>303</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>304</v>
-      </c>
-      <c r="E56" t="s">
-        <v>305</v>
       </c>
       <c r="F56" t="s">
         <v>32</v>
       </c>
       <c r="G56" t="s">
-        <v>306</v>
-      </c>
-      <c r="H56" t="s">
-        <v>14</v>
+        <v>251</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
+        <v>305</v>
+      </c>
+      <c r="B57" t="s">
+        <v>291</v>
+      </c>
+      <c r="C57" t="s">
+        <v>306</v>
+      </c>
+      <c r="D57" t="s">
         <v>307</v>
       </c>
-      <c r="B57" t="s">
-        <v>297</v>
-      </c>
-      <c r="C57" t="s">
+      <c r="E57" t="s">
         <v>308</v>
-      </c>
-      <c r="D57" t="s">
-        <v>309</v>
-      </c>
-      <c r="E57" t="s">
-        <v>310</v>
       </c>
       <c r="F57" t="s">
         <v>32</v>
       </c>
       <c r="G57" t="s">
-        <v>257</v>
-      </c>
-      <c r="H57" t="s">
-        <v>14</v>
+        <v>261</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
+        <v>309</v>
+      </c>
+      <c r="B58" t="s">
+        <v>310</v>
+      </c>
+      <c r="C58" t="s">
         <v>311</v>
       </c>
-      <c r="B58" t="s">
-        <v>297</v>
-      </c>
-      <c r="C58" t="s">
+      <c r="D58" t="s">
         <v>312</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>313</v>
       </c>
-      <c r="E58" t="s">
+      <c r="F58" t="s">
+        <v>103</v>
+      </c>
+      <c r="G58" t="s">
         <v>314</v>
       </c>
-      <c r="F58" t="s">
-        <v>32</v>
-      </c>
-      <c r="G58" t="s">
-        <v>267</v>
-      </c>
-      <c r="H58" t="s">
-        <v>14</v>
+      <c r="H58" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3620,16 +3614,16 @@
         <v>319</v>
       </c>
       <c r="F59" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="G59" t="s">
         <v>320</v>
       </c>
-      <c r="H59" t="s">
-        <v>14</v>
+      <c r="H59" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3637,36 +3631,36 @@
         <v>321</v>
       </c>
       <c r="B60" t="s">
+        <v>316</v>
+      </c>
+      <c r="C60" t="s">
         <v>322</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>323</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>324</v>
-      </c>
-      <c r="E60" t="s">
-        <v>325</v>
       </c>
       <c r="F60" t="s">
         <v>53</v>
       </c>
       <c r="G60" t="s">
-        <v>326</v>
-      </c>
-      <c r="H60" t="s">
-        <v>14</v>
+        <v>325</v>
+      </c>
+      <c r="H60" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
+        <v>326</v>
+      </c>
+      <c r="B61" t="s">
         <v>327</v>
-      </c>
-      <c r="B61" t="s">
-        <v>322</v>
       </c>
       <c r="C61" t="s">
         <v>328</v>
@@ -3683,11 +3677,11 @@
       <c r="G61" t="s">
         <v>331</v>
       </c>
-      <c r="H61" t="s">
-        <v>14</v>
+      <c r="H61" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="62" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3695,57 +3689,57 @@
         <v>332</v>
       </c>
       <c r="B62" t="s">
+        <v>327</v>
+      </c>
+      <c r="C62" t="s">
         <v>333</v>
       </c>
-      <c r="C62" t="s">
+      <c r="D62" t="s">
         <v>334</v>
       </c>
-      <c r="D62" t="s">
+      <c r="E62" t="s">
         <v>335</v>
       </c>
-      <c r="E62" t="s">
-        <v>336</v>
-      </c>
       <c r="F62" t="s">
-        <v>53</v>
+        <v>103</v>
       </c>
       <c r="G62" t="s">
-        <v>337</v>
-      </c>
-      <c r="H62" t="s">
-        <v>14</v>
+        <v>125</v>
+      </c>
+      <c r="H62" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
+        <v>336</v>
+      </c>
+      <c r="B63" t="s">
+        <v>337</v>
+      </c>
+      <c r="C63" t="s">
         <v>338</v>
       </c>
-      <c r="B63" t="s">
-        <v>333</v>
-      </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
         <v>339</v>
       </c>
-      <c r="D63" t="s">
+      <c r="E63" t="s">
         <v>340</v>
-      </c>
-      <c r="E63" t="s">
-        <v>341</v>
       </c>
       <c r="F63" t="s">
         <v>103</v>
       </c>
       <c r="G63" t="s">
-        <v>125</v>
-      </c>
-      <c r="H63" t="s">
-        <v>14</v>
+        <v>341</v>
+      </c>
+      <c r="H63" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3765,16 +3759,16 @@
         <v>346</v>
       </c>
       <c r="F64" t="s">
-        <v>103</v>
+        <v>32</v>
       </c>
       <c r="G64" t="s">
         <v>347</v>
       </c>
-      <c r="H64" t="s">
-        <v>14</v>
+      <c r="H64" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3782,65 +3776,65 @@
         <v>348</v>
       </c>
       <c r="B65" t="s">
+        <v>343</v>
+      </c>
+      <c r="C65" t="s">
         <v>349</v>
       </c>
-      <c r="C65" t="s">
+      <c r="D65" t="s">
         <v>350</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>351</v>
-      </c>
-      <c r="E65" t="s">
-        <v>352</v>
       </c>
       <c r="F65" t="s">
         <v>32</v>
       </c>
       <c r="G65" t="s">
-        <v>353</v>
-      </c>
-      <c r="H65" t="s">
-        <v>14</v>
+        <v>352</v>
+      </c>
+      <c r="H65" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="66" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
+        <v>353</v>
+      </c>
+      <c r="B66" t="s">
+        <v>343</v>
+      </c>
+      <c r="C66" t="s">
         <v>354</v>
       </c>
-      <c r="B66" t="s">
-        <v>349</v>
-      </c>
-      <c r="C66" t="s">
+      <c r="D66" t="s">
         <v>355</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" t="s">
         <v>356</v>
       </c>
-      <c r="E66" t="s">
+      <c r="F66" t="s">
+        <v>53</v>
+      </c>
+      <c r="G66" t="s">
         <v>357</v>
       </c>
-      <c r="F66" t="s">
-        <v>32</v>
-      </c>
-      <c r="G66" t="s">
-        <v>358</v>
-      </c>
-      <c r="H66" t="s">
-        <v>14</v>
+      <c r="H66" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="67" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
+        <v>358</v>
+      </c>
+      <c r="B67" t="s">
         <v>359</v>
-      </c>
-      <c r="B67" t="s">
-        <v>349</v>
       </c>
       <c r="C67" t="s">
         <v>360</v>
@@ -3852,16 +3846,16 @@
         <v>362</v>
       </c>
       <c r="F67" t="s">
-        <v>53</v>
+        <v>103</v>
       </c>
       <c r="G67" t="s">
         <v>363</v>
       </c>
-      <c r="H67" t="s">
-        <v>14</v>
+      <c r="H67" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3886,11 +3880,11 @@
       <c r="G68" t="s">
         <v>369</v>
       </c>
-      <c r="H68" t="s">
-        <v>14</v>
+      <c r="H68" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3910,16 +3904,16 @@
         <v>374</v>
       </c>
       <c r="F69" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="G69" t="s">
         <v>375</v>
       </c>
-      <c r="H69" t="s">
-        <v>14</v>
+      <c r="H69" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3927,94 +3921,94 @@
         <v>376</v>
       </c>
       <c r="B70" t="s">
+        <v>371</v>
+      </c>
+      <c r="C70" t="s">
         <v>377</v>
       </c>
-      <c r="C70" t="s">
+      <c r="D70" t="s">
         <v>378</v>
       </c>
-      <c r="D70" t="s">
+      <c r="E70" t="s">
         <v>379</v>
-      </c>
-      <c r="E70" t="s">
-        <v>380</v>
       </c>
       <c r="F70" t="s">
         <v>53</v>
       </c>
       <c r="G70" t="s">
-        <v>381</v>
-      </c>
-      <c r="H70" t="s">
-        <v>14</v>
+        <v>375</v>
+      </c>
+      <c r="H70" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
+        <v>380</v>
+      </c>
+      <c r="B71" t="s">
+        <v>371</v>
+      </c>
+      <c r="C71" t="s">
+        <v>381</v>
+      </c>
+      <c r="D71" t="s">
         <v>382</v>
       </c>
-      <c r="B71" t="s">
-        <v>377</v>
-      </c>
-      <c r="C71" t="s">
+      <c r="E71" t="s">
         <v>383</v>
-      </c>
-      <c r="D71" t="s">
-        <v>384</v>
-      </c>
-      <c r="E71" t="s">
-        <v>385</v>
       </c>
       <c r="F71" t="s">
         <v>53</v>
       </c>
       <c r="G71" t="s">
-        <v>381</v>
-      </c>
-      <c r="H71" t="s">
-        <v>14</v>
+        <v>384</v>
+      </c>
+      <c r="H71" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I71" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
+        <v>385</v>
+      </c>
+      <c r="B72" t="s">
+        <v>371</v>
+      </c>
+      <c r="C72" t="s">
         <v>386</v>
       </c>
-      <c r="B72" t="s">
-        <v>377</v>
-      </c>
-      <c r="C72" t="s">
+      <c r="D72" t="s">
         <v>387</v>
       </c>
-      <c r="D72" t="s">
+      <c r="E72" t="s">
         <v>388</v>
       </c>
-      <c r="E72" t="s">
+      <c r="F72" t="s">
+        <v>103</v>
+      </c>
+      <c r="G72" t="s">
         <v>389</v>
       </c>
-      <c r="F72" t="s">
-        <v>53</v>
-      </c>
-      <c r="G72" t="s">
-        <v>390</v>
-      </c>
-      <c r="H72" t="s">
-        <v>14</v>
+      <c r="H72" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="73" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
+        <v>390</v>
+      </c>
+      <c r="B73" t="s">
         <v>391</v>
-      </c>
-      <c r="B73" t="s">
-        <v>377</v>
       </c>
       <c r="C73" t="s">
         <v>392</v>
@@ -4026,16 +4020,16 @@
         <v>394</v>
       </c>
       <c r="F73" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="G73" t="s">
         <v>395</v>
       </c>
-      <c r="H73" t="s">
-        <v>14</v>
+      <c r="H73" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -4043,65 +4037,65 @@
         <v>396</v>
       </c>
       <c r="B74" t="s">
+        <v>391</v>
+      </c>
+      <c r="C74" t="s">
         <v>397</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D74" t="s">
         <v>398</v>
       </c>
-      <c r="D74" t="s">
+      <c r="E74" t="s">
         <v>399</v>
-      </c>
-      <c r="E74" t="s">
-        <v>400</v>
       </c>
       <c r="F74" t="s">
         <v>53</v>
       </c>
       <c r="G74" t="s">
-        <v>401</v>
-      </c>
-      <c r="H74" t="s">
-        <v>14</v>
+        <v>98</v>
+      </c>
+      <c r="H74" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="75" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
+        <v>400</v>
+      </c>
+      <c r="B75" t="s">
+        <v>391</v>
+      </c>
+      <c r="C75" t="s">
+        <v>401</v>
+      </c>
+      <c r="D75" t="s">
         <v>402</v>
       </c>
-      <c r="B75" t="s">
-        <v>397</v>
-      </c>
-      <c r="C75" t="s">
+      <c r="E75" t="s">
         <v>403</v>
-      </c>
-      <c r="D75" t="s">
-        <v>404</v>
-      </c>
-      <c r="E75" t="s">
-        <v>405</v>
       </c>
       <c r="F75" t="s">
         <v>53</v>
       </c>
       <c r="G75" t="s">
-        <v>98</v>
-      </c>
-      <c r="H75" t="s">
-        <v>14</v>
+        <v>404</v>
+      </c>
+      <c r="H75" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
+        <v>405</v>
+      </c>
+      <c r="B76" t="s">
         <v>406</v>
-      </c>
-      <c r="B76" t="s">
-        <v>397</v>
       </c>
       <c r="C76" t="s">
         <v>407</v>
@@ -4113,16 +4107,16 @@
         <v>409</v>
       </c>
       <c r="F76" t="s">
-        <v>53</v>
+        <v>103</v>
       </c>
       <c r="G76" t="s">
         <v>410</v>
       </c>
-      <c r="H76" t="s">
-        <v>14</v>
+      <c r="H76" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -4130,36 +4124,36 @@
         <v>411</v>
       </c>
       <c r="B77" t="s">
+        <v>406</v>
+      </c>
+      <c r="C77" t="s">
         <v>412</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D77" t="s">
         <v>413</v>
       </c>
-      <c r="D77" t="s">
+      <c r="E77" t="s">
         <v>414</v>
-      </c>
-      <c r="E77" t="s">
-        <v>415</v>
       </c>
       <c r="F77" t="s">
         <v>103</v>
       </c>
       <c r="G77" t="s">
-        <v>416</v>
-      </c>
-      <c r="H77" t="s">
-        <v>14</v>
+        <v>415</v>
+      </c>
+      <c r="H77" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I77" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="78" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
+        <v>416</v>
+      </c>
+      <c r="B78" t="s">
         <v>417</v>
-      </c>
-      <c r="B78" t="s">
-        <v>412</v>
       </c>
       <c r="C78" t="s">
         <v>418</v>
@@ -4171,16 +4165,16 @@
         <v>420</v>
       </c>
       <c r="F78" t="s">
-        <v>103</v>
+        <v>32</v>
       </c>
       <c r="G78" t="s">
         <v>421</v>
       </c>
-      <c r="H78" t="s">
-        <v>14</v>
+      <c r="H78" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -4188,92 +4182,63 @@
         <v>422</v>
       </c>
       <c r="B79" t="s">
+        <v>417</v>
+      </c>
+      <c r="C79" t="s">
         <v>423</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D79" t="s">
         <v>424</v>
       </c>
-      <c r="D79" t="s">
+      <c r="E79" t="s">
         <v>425</v>
       </c>
-      <c r="E79" t="s">
+      <c r="F79" t="s">
+        <v>53</v>
+      </c>
+      <c r="G79" t="s">
         <v>426</v>
       </c>
-      <c r="F79" t="s">
-        <v>32</v>
-      </c>
-      <c r="G79" t="s">
-        <v>427</v>
-      </c>
-      <c r="H79" t="s">
-        <v>14</v>
+      <c r="H79" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
+        <v>427</v>
+      </c>
+      <c r="B80" t="s">
+        <v>417</v>
+      </c>
+      <c r="C80" t="s">
         <v>428</v>
       </c>
-      <c r="B80" t="s">
-        <v>423</v>
-      </c>
-      <c r="C80" t="s">
+      <c r="D80" t="s">
         <v>429</v>
       </c>
-      <c r="D80" t="s">
+      <c r="E80" t="s">
         <v>430</v>
-      </c>
-      <c r="E80" t="s">
-        <v>431</v>
       </c>
       <c r="F80" t="s">
         <v>53</v>
       </c>
       <c r="G80" t="s">
-        <v>432</v>
-      </c>
-      <c r="H80" t="s">
-        <v>14</v>
+        <v>431</v>
+      </c>
+      <c r="H80" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
-        <v>433</v>
-      </c>
-      <c r="B81" t="s">
-        <v>423</v>
-      </c>
-      <c r="C81" t="s">
-        <v>434</v>
-      </c>
-      <c r="D81" t="s">
-        <v>435</v>
-      </c>
-      <c r="E81" t="s">
-        <v>436</v>
-      </c>
-      <c r="F81" t="s">
-        <v>53</v>
-      </c>
-      <c r="G81" t="s">
-        <v>437</v>
-      </c>
-      <c r="H81" t="s">
-        <v>14</v>
-      </c>
-      <c r="I81" s="3" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K81" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:K80" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H81" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H80" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Not Started,Pass,Fail,N/A,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4299,7 +4264,7 @@
         <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -4310,7 +4275,7 @@
         <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -4321,7 +4286,7 @@
         <v>53</v>
       </c>
       <c r="C3" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -4332,7 +4297,7 @@
         <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -4340,10 +4305,10 @@
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="C5" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -4351,7 +4316,7 @@
         <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>